<commit_message>
DCA + Calibration Curve fixed.
</commit_message>
<xml_diff>
--- a/Single/publication_plots_single/supplementary_model_selection_table.xlsx
+++ b/Single/publication_plots_single/supplementary_model_selection_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
   <si>
     <t>Dataset</t>
   </si>
@@ -70,22 +70,25 @@
     <t>ADC_M1</t>
   </si>
   <si>
+    <t>mrmr_then_elasticnet_no_corr_auto_k_smote</t>
+  </si>
+  <si>
+    <t>mrmr_then_elasticnet_no_corr_auto_k_no_smote</t>
+  </si>
+  <si>
+    <t>elasticnet_then_mrmr_auto_k_smote</t>
+  </si>
+  <si>
+    <t>corr_mrmr_auto_k_no_smote</t>
+  </si>
+  <si>
+    <t>corr_mrmr_auto_k_smote</t>
+  </si>
+  <si>
     <t>elasticnet_then_mrmr_auto_k_no_smote</t>
   </si>
   <si>
-    <t>elasticnet_then_mrmr_auto_k_smote</t>
-  </si>
-  <si>
-    <t>corr_mrmr_auto_k_no_smote</t>
-  </si>
-  <si>
-    <t>corr_mrmr_auto_k_smote</t>
-  </si>
-  <si>
-    <t>mrmr_then_elasticnet_no_corr_auto_k_no_smote</t>
-  </si>
-  <si>
-    <t>mrmr_then_elasticnet_no_corr_auto_k_smote</t>
+    <t>mrmr_then_elasticnet_no_corr</t>
   </si>
   <si>
     <t>elasticnet_then_mrmr</t>
@@ -94,19 +97,19 @@
     <t>corr_mrmr</t>
   </si>
   <si>
-    <t>mrmr_then_elasticnet_no_corr</t>
-  </si>
-  <si>
     <t>auto</t>
   </si>
   <si>
+    <t>SVM_Linear</t>
+  </si>
+  <si>
     <t>LogisticRegression</t>
   </si>
   <si>
-    <t>SVM_Linear</t>
-  </si>
-  <si>
-    <t>SVM_RBF</t>
+    <t>LightGBM</t>
+  </si>
+  <si>
+    <t>KNN</t>
   </si>
 </sst>
 </file>
@@ -534,43 +537,43 @@
         <v>27</v>
       </c>
       <c r="E2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="s">
         <v>28</v>
       </c>
       <c r="G2">
-        <v>0.771</v>
+        <v>0.764</v>
       </c>
       <c r="H2">
-        <v>0.038</v>
+        <v>0.08</v>
       </c>
       <c r="I2">
-        <v>0.71</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="J2">
-        <v>0.8090000000000001</v>
+        <v>0.799</v>
       </c>
       <c r="K2">
-        <v>0.743</v>
+        <v>0.72</v>
       </c>
       <c r="L2">
-        <v>0.6870000000000001</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="M2">
-        <v>0.672</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="N2">
-        <v>0.66</v>
+        <v>0.671</v>
       </c>
       <c r="O2">
-        <v>0.678</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="P2">
-        <v>14.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Q2">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -587,43 +590,43 @@
         <v>27</v>
       </c>
       <c r="E3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
       </c>
       <c r="G3">
-        <v>0.764</v>
+        <v>0.762</v>
       </c>
       <c r="H3">
-        <v>0.051</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="I3">
-        <v>0.72</v>
+        <v>0.715</v>
       </c>
       <c r="J3">
         <v>0.8159999999999999</v>
       </c>
       <c r="K3">
-        <v>0.738</v>
+        <v>0.758</v>
       </c>
       <c r="L3">
-        <v>0.701</v>
+        <v>0.714</v>
       </c>
       <c r="M3">
-        <v>0.6899999999999999</v>
+        <v>0.698</v>
       </c>
       <c r="N3">
-        <v>0.6850000000000001</v>
+        <v>0.6860000000000001</v>
       </c>
       <c r="O3">
-        <v>0.695</v>
+        <v>0.706</v>
       </c>
       <c r="P3">
-        <v>14.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Q3">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -640,43 +643,43 @@
         <v>27</v>
       </c>
       <c r="E4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G4">
-        <v>0.745</v>
+        <v>0.76</v>
       </c>
       <c r="H4">
-        <v>0.026</v>
+        <v>0.06</v>
       </c>
       <c r="I4">
-        <v>0.696</v>
+        <v>0.726</v>
       </c>
       <c r="J4">
-        <v>0.797</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="K4">
-        <v>0.759</v>
+        <v>0.766</v>
       </c>
       <c r="L4">
-        <v>0.6879999999999999</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="M4">
-        <v>0.67</v>
+        <v>0.664</v>
       </c>
       <c r="N4">
-        <v>0.669</v>
+        <v>0.701</v>
       </c>
       <c r="O4">
-        <v>0.6830000000000001</v>
+        <v>0.698</v>
       </c>
       <c r="P4">
-        <v>12.8</v>
+        <v>13.2</v>
       </c>
       <c r="Q4">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -687,49 +690,49 @@
         <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
         <v>27</v>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G5">
-        <v>0.744</v>
+        <v>0.748</v>
       </c>
       <c r="H5">
-        <v>0.028</v>
+        <v>0.026</v>
       </c>
       <c r="I5">
-        <v>0.694</v>
+        <v>0.703</v>
       </c>
       <c r="J5">
-        <v>0.804</v>
+        <v>0.802</v>
       </c>
       <c r="K5">
-        <v>0.761</v>
+        <v>0.764</v>
       </c>
       <c r="L5">
-        <v>0.681</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="M5">
-        <v>0.662</v>
+        <v>0.672</v>
       </c>
       <c r="N5">
-        <v>0.661</v>
+        <v>0.669</v>
       </c>
       <c r="O5">
-        <v>0.672</v>
+        <v>0.678</v>
       </c>
       <c r="P5">
-        <v>12.8</v>
+        <v>12</v>
       </c>
       <c r="Q5">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -746,43 +749,43 @@
         <v>27</v>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G6">
-        <v>0.711</v>
+        <v>0.732</v>
       </c>
       <c r="H6">
-        <v>0.075</v>
+        <v>0.032</v>
       </c>
       <c r="I6">
-        <v>0.694</v>
+        <v>0.696</v>
       </c>
       <c r="J6">
-        <v>0.77</v>
+        <v>0.796</v>
       </c>
       <c r="K6">
-        <v>0.729</v>
+        <v>0.758</v>
       </c>
       <c r="L6">
-        <v>0.6919999999999999</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="M6">
-        <v>0.68</v>
+        <v>0.668</v>
       </c>
       <c r="N6">
-        <v>0.6870000000000001</v>
+        <v>0.681</v>
       </c>
       <c r="O6">
         <v>0.6889999999999999</v>
       </c>
       <c r="P6">
-        <v>12.4</v>
+        <v>12</v>
       </c>
       <c r="Q6">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -793,49 +796,49 @@
         <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
         <v>27</v>
       </c>
       <c r="E7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G7">
-        <v>0.697</v>
+        <v>0.728</v>
       </c>
       <c r="H7">
-        <v>0.026</v>
+        <v>0.041</v>
       </c>
       <c r="I7">
-        <v>0.671</v>
+        <v>0.668</v>
       </c>
       <c r="J7">
-        <v>0.767</v>
+        <v>0.745</v>
       </c>
       <c r="K7">
-        <v>0.706</v>
+        <v>0.699</v>
       </c>
       <c r="L7">
-        <v>0.633</v>
+        <v>0.681</v>
       </c>
       <c r="M7">
-        <v>0.644</v>
+        <v>0.666</v>
       </c>
       <c r="N7">
-        <v>0.665</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="O7">
-        <v>0.6879999999999999</v>
+        <v>0.694</v>
       </c>
       <c r="P7">
-        <v>12.4</v>
+        <v>13.2</v>
       </c>
       <c r="Q7">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Plots added and some stuffs fixed.
</commit_message>
<xml_diff>
--- a/Single/publication_plots_single/supplementary_model_selection_table.xlsx
+++ b/Single/publication_plots_single/supplementary_model_selection_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="54">
   <si>
     <t>Dataset</t>
   </si>
@@ -65,6 +65,72 @@
   </si>
   <si>
     <t>N_Unique_Selected_Features</t>
+  </si>
+  <si>
+    <t>Mean_Kappa</t>
+  </si>
+  <si>
+    <t>Std_Kappa</t>
+  </si>
+  <si>
+    <t>Pooled_Kappa</t>
+  </si>
+  <si>
+    <t>Pooled_Kappa_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_Kappa_CI95_High</t>
+  </si>
+  <si>
+    <t>Pooled_AUC_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_AUC_CI95_High</t>
+  </si>
+  <si>
+    <t>Pooled_PR_AUC_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_PR_AUC_CI95_High</t>
+  </si>
+  <si>
+    <t>Pooled_Acc_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_Acc_CI95_High</t>
+  </si>
+  <si>
+    <t>Pooled_Bal_Acc_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_Bal_Acc_CI95_High</t>
+  </si>
+  <si>
+    <t>Pooled_F1_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_F1_CI95_High</t>
+  </si>
+  <si>
+    <t>Pooled_Rec_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_Rec_CI95_High</t>
+  </si>
+  <si>
+    <t>Pooled_Specificity_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_Specificity_CI95_High</t>
+  </si>
+  <si>
+    <t>Pooled_Brier</t>
+  </si>
+  <si>
+    <t>Pooled_Brier_CI95_Low</t>
+  </si>
+  <si>
+    <t>Pooled_Brier_CI95_High</t>
   </si>
   <si>
     <t>ADC_M1</t>
@@ -467,10 +533,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:AM7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:39">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -522,25 +588,91 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:39">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="G2">
         <v>0.764</v>
@@ -575,25 +707,91 @@
       <c r="Q2">
         <v>29</v>
       </c>
+      <c r="R2">
+        <v>0.367</v>
+      </c>
+      <c r="S2">
+        <v>0.131</v>
+      </c>
+      <c r="T2">
+        <v>0.356</v>
+      </c>
+      <c r="U2">
+        <v>0.165</v>
+      </c>
+      <c r="V2">
+        <v>0.525</v>
+      </c>
+      <c r="W2">
+        <v>0.5629999999999999</v>
+      </c>
+      <c r="X2">
+        <v>0.8090000000000001</v>
+      </c>
+      <c r="Y2">
+        <v>0.513</v>
+      </c>
+      <c r="Z2">
+        <v>0.894</v>
+      </c>
+      <c r="AA2">
+        <v>0.581</v>
+      </c>
+      <c r="AB2">
+        <v>0.765</v>
+      </c>
+      <c r="AC2">
+        <v>0.585</v>
+      </c>
+      <c r="AD2">
+        <v>0.775</v>
+      </c>
+      <c r="AE2">
+        <v>0.533</v>
+      </c>
+      <c r="AF2">
+        <v>0.797</v>
+      </c>
+      <c r="AG2">
+        <v>0.477</v>
+      </c>
+      <c r="AH2">
+        <v>0.761</v>
+      </c>
+      <c r="AI2">
+        <v>0.604</v>
+      </c>
+      <c r="AJ2">
+        <v>0.87</v>
+      </c>
+      <c r="AK2">
+        <v>0.229</v>
+      </c>
+      <c r="AL2">
+        <v>0.189</v>
+      </c>
+      <c r="AM2">
+        <v>0.274</v>
+      </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:39">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="G3">
         <v>0.762</v>
@@ -628,25 +826,91 @@
       <c r="Q3">
         <v>29</v>
       </c>
+      <c r="R3">
+        <v>0.401</v>
+      </c>
+      <c r="S3">
+        <v>0.121</v>
+      </c>
+      <c r="T3">
+        <v>0.389</v>
+      </c>
+      <c r="U3">
+        <v>0.199</v>
+      </c>
+      <c r="V3">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="W3">
+        <v>0.592</v>
+      </c>
+      <c r="X3">
+        <v>0.832</v>
+      </c>
+      <c r="Y3">
+        <v>0.5590000000000001</v>
+      </c>
+      <c r="Z3">
+        <v>0.907</v>
+      </c>
+      <c r="AA3">
+        <v>0.6</v>
+      </c>
+      <c r="AB3">
+        <v>0.783</v>
+      </c>
+      <c r="AC3">
+        <v>0.603</v>
+      </c>
+      <c r="AD3">
+        <v>0.79</v>
+      </c>
+      <c r="AE3">
+        <v>0.554</v>
+      </c>
+      <c r="AF3">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="AG3">
+        <v>0.5</v>
+      </c>
+      <c r="AH3">
+        <v>0.786</v>
+      </c>
+      <c r="AI3">
+        <v>0.607</v>
+      </c>
+      <c r="AJ3">
+        <v>0.878</v>
+      </c>
+      <c r="AK3">
+        <v>0.217</v>
+      </c>
+      <c r="AL3">
+        <v>0.178</v>
+      </c>
+      <c r="AM3">
+        <v>0.258</v>
+      </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:39">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="G4">
         <v>0.76</v>
@@ -681,25 +945,91 @@
       <c r="Q4">
         <v>27</v>
       </c>
+      <c r="R4">
+        <v>0.362</v>
+      </c>
+      <c r="S4">
+        <v>0.178</v>
+      </c>
+      <c r="T4">
+        <v>0.326</v>
+      </c>
+      <c r="U4">
+        <v>0.116</v>
+      </c>
+      <c r="V4">
+        <v>0.521</v>
+      </c>
+      <c r="W4">
+        <v>0.607</v>
+      </c>
+      <c r="X4">
+        <v>0.836</v>
+      </c>
+      <c r="Y4">
+        <v>0.583</v>
+      </c>
+      <c r="Z4">
+        <v>0.894</v>
+      </c>
+      <c r="AA4">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AB4">
+        <v>0.769</v>
+      </c>
+      <c r="AC4">
+        <v>0.5590000000000001</v>
+      </c>
+      <c r="AD4">
+        <v>0.766</v>
+      </c>
+      <c r="AE4">
+        <v>0.545</v>
+      </c>
+      <c r="AF4">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="AG4">
+        <v>0.528</v>
+      </c>
+      <c r="AH4">
+        <v>0.829</v>
+      </c>
+      <c r="AI4">
+        <v>0.486</v>
+      </c>
+      <c r="AJ4">
+        <v>0.795</v>
+      </c>
+      <c r="AK4">
+        <v>0.238</v>
+      </c>
+      <c r="AL4">
+        <v>0.172</v>
+      </c>
+      <c r="AM4">
+        <v>0.306</v>
+      </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:39">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="G5">
         <v>0.748</v>
@@ -734,25 +1064,91 @@
       <c r="Q5">
         <v>36</v>
       </c>
+      <c r="R5">
+        <v>0.366</v>
+      </c>
+      <c r="S5">
+        <v>0.131</v>
+      </c>
+      <c r="T5">
+        <v>0.338</v>
+      </c>
+      <c r="U5">
+        <v>0.125</v>
+      </c>
+      <c r="V5">
+        <v>0.532</v>
+      </c>
+      <c r="W5">
+        <v>0.583</v>
+      </c>
+      <c r="X5">
+        <v>0.8159999999999999</v>
+      </c>
+      <c r="Y5">
+        <v>0.579</v>
+      </c>
+      <c r="Z5">
+        <v>0.899</v>
+      </c>
+      <c r="AA5">
+        <v>0.5620000000000001</v>
+      </c>
+      <c r="AB5">
+        <v>0.767</v>
+      </c>
+      <c r="AC5">
+        <v>0.5649999999999999</v>
+      </c>
+      <c r="AD5">
+        <v>0.772</v>
+      </c>
+      <c r="AE5">
+        <v>0.516</v>
+      </c>
+      <c r="AF5">
+        <v>0.796</v>
+      </c>
+      <c r="AG5">
+        <v>0.452</v>
+      </c>
+      <c r="AH5">
+        <v>0.784</v>
+      </c>
+      <c r="AI5">
+        <v>0.5659999999999999</v>
+      </c>
+      <c r="AJ5">
+        <v>0.854</v>
+      </c>
+      <c r="AK5">
+        <v>0.221</v>
+      </c>
+      <c r="AL5">
+        <v>0.19</v>
+      </c>
+      <c r="AM5">
+        <v>0.252</v>
+      </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:39">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="G6">
         <v>0.732</v>
@@ -787,25 +1183,91 @@
       <c r="Q6">
         <v>36</v>
       </c>
+      <c r="R6">
+        <v>0.358</v>
+      </c>
+      <c r="S6">
+        <v>0.105</v>
+      </c>
+      <c r="T6">
+        <v>0.332</v>
+      </c>
+      <c r="U6">
+        <v>0.132</v>
+      </c>
+      <c r="V6">
+        <v>0.522</v>
+      </c>
+      <c r="W6">
+        <v>0.58</v>
+      </c>
+      <c r="X6">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="Y6">
+        <v>0.569</v>
+      </c>
+      <c r="Z6">
+        <v>0.893</v>
+      </c>
+      <c r="AA6">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="AB6">
+        <v>0.767</v>
+      </c>
+      <c r="AC6">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="AD6">
+        <v>0.77</v>
+      </c>
+      <c r="AE6">
+        <v>0.543</v>
+      </c>
+      <c r="AF6">
+        <v>0.803</v>
+      </c>
+      <c r="AG6">
+        <v>0.5</v>
+      </c>
+      <c r="AH6">
+        <v>0.8</v>
+      </c>
+      <c r="AI6">
+        <v>0.52</v>
+      </c>
+      <c r="AJ6">
+        <v>0.833</v>
+      </c>
+      <c r="AK6">
+        <v>0.226</v>
+      </c>
+      <c r="AL6">
+        <v>0.194</v>
+      </c>
+      <c r="AM6">
+        <v>0.26</v>
+      </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:39">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="G7">
         <v>0.728</v>
@@ -839,6 +1301,72 @@
       </c>
       <c r="Q7">
         <v>27</v>
+      </c>
+      <c r="R7">
+        <v>0.34</v>
+      </c>
+      <c r="S7">
+        <v>0.115</v>
+      </c>
+      <c r="T7">
+        <v>0.329</v>
+      </c>
+      <c r="U7">
+        <v>0.133</v>
+      </c>
+      <c r="V7">
+        <v>0.512</v>
+      </c>
+      <c r="W7">
+        <v>0.541</v>
+      </c>
+      <c r="X7">
+        <v>0.783</v>
+      </c>
+      <c r="Y7">
+        <v>0.504</v>
+      </c>
+      <c r="Z7">
+        <v>0.849</v>
+      </c>
+      <c r="AA7">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="AB7">
+        <v>0.763</v>
+      </c>
+      <c r="AC7">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="AD7">
+        <v>0.761</v>
+      </c>
+      <c r="AE7">
+        <v>0.539</v>
+      </c>
+      <c r="AF7">
+        <v>0.8</v>
+      </c>
+      <c r="AG7">
+        <v>0.521</v>
+      </c>
+      <c r="AH7">
+        <v>0.805</v>
+      </c>
+      <c r="AI7">
+        <v>0.509</v>
+      </c>
+      <c r="AJ7">
+        <v>0.804</v>
+      </c>
+      <c r="AK7">
+        <v>0.236</v>
+      </c>
+      <c r="AL7">
+        <v>0.187</v>
+      </c>
+      <c r="AM7">
+        <v>0.289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>